<commit_message>
add 8B in Table3
</commit_message>
<xml_diff>
--- a/eval/results/statistical_tests_new30.xlsx
+++ b/eval/results/statistical_tests_new30.xlsx
@@ -16682,7 +16682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16777,6 +16777,231 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Llama3.1-8B</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>82.6</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>85.7</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>85.7</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>79.2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>100.0*†</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Llama3.1-8B</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>90.0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>42.9</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>66.7</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>85.7**</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Llama3.1-8B</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>81.8</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>90.9</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>78.3</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>47.4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>52.6</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>94.7**</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Llama3.1-8B</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>83.3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>85.7</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>52.6</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>52.6</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>94.7**</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Llama3.1-8B</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>14</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>81.2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>90.9</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>86.4</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>95.0*†</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>